<commit_message>
update seed temas and update seed acoes - tinha uma acao com numero repetido
</commit_message>
<xml_diff>
--- a/backend/estrutura_pdm/data/xl/dados_metas_atualizados_v2.xlsx
+++ b/backend/estrutura_pdm/data/xl/dados_metas_atualizados_v2.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2749" uniqueCount="1464">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2749" uniqueCount="1465">
   <si>
     <t>Número da Meta</t>
   </si>
@@ -4536,6 +4536,9 @@
   </si>
   <si>
     <t>O eixo Capital do Futuro reúne metas voltadas à modernização da administração pública, à transformação digital e ao aperfeiçoamento da relação entre governo e cidadão. Trata do compromisso com a transparência e da participação das pessoas como protagonistas dos processos decisórios.</t>
+  </si>
+  <si>
+    <t>129.04</t>
   </si>
 </sst>
 </file>
@@ -5599,7 +5602,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -16365,7 +16368,7 @@
         <v>1428</v>
       </c>
       <c r="C342" t="s">
-        <v>1433</v>
+        <v>1464</v>
       </c>
       <c r="D342" t="s">
         <v>1435</v>
@@ -16631,6 +16634,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100506FD4652602C740A483E9D3DF6A153B" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3ae790dad332779219ad741447ce1449">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1aa39b8c-19b3-4ca5-9ada-a1970df5e875" xmlns:ns3="a9968193-2d77-4b73-840a-26fc33ae728b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="bceb73c01ba1e25437ffc1b7a59fee3b" ns2:_="" ns3:_="">
     <xsd:import namespace="1aa39b8c-19b3-4ca5-9ada-a1970df5e875"/>
@@ -16885,15 +16897,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -16906,6 +16909,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2FD2D9B6-68AB-4A59-BCBA-EC7E4F0054ED}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9BFC49B3-58DA-49B8-A3A9-093E89BDDE73}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -16924,14 +16935,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2FD2D9B6-68AB-4A59-BCBA-EC7E4F0054ED}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B9DFCD87-1494-4CF4-9D60-842DA5D97CB7}">
   <ds:schemaRefs>

</xml_diff>